<commit_message>
docs: record V5 G2 repair review checkpoint
</commit_message>
<xml_diff>
--- a/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
+++ b/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="R10a334a637d84fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="R0d0bcc245cfd4cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="R2eb298ea80d04c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="Rd8cace3c3a7d405f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="Rd421f395adcb44d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="Re1e6f756080144d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R681f35692dad42d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="Ra0821498851b497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="Rbe6338754f834388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Rae8c467c74ec4615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="R5e2337de7ea14b19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="R9fa1011a8f9942c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="R31c2e34f4aaa4163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="Rf1ceb51e07ec4956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="R668369dab1b840e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="Ra64fa2bca96d4324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="Rcaf24e6c79484f7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="R4a709ec37def4922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="R58828281026940f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R3a07347bd81c486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="R423920dbf7954ca9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="R24f79f6a08234299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Ra16b2318e28f4718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="Re876932919c8454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="Rb8e9cf8ee00448a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="R4a772bc04b564fc0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25665,7 +25665,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>1.0.0-v5-g2-runtime-candidate-001</x:v>
+        <x:v>1.0.1-v5-g2-repair-001</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
         <x:v>6</x:v>
@@ -25705,7 +25705,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 IMPLEMENTED_PENDING_INDEPENDENT_REVIEW</x:v>
+        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
         <x:v>13</x:v>
@@ -25724,7 +25724,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>独立复审 V5-G2 runtime candidate；复审前不得进入 G3/G4/V6</x:v>
+        <x:v>由全新 reviewer 独立复审 V5-G2 repair candidate；复审前不得进入 G3/G4/G5/G6/V6</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
         <x:v>15</x:v>
@@ -26838,6 +26838,44 @@
         <x:v>1100</x:v>
       </x:c>
     </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>RISK-012</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Risk</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>V2 aggregate validator 若只检查 next sequence 为正而不高于既有 stable ID，冷恢复后的新训练/派遣会复用 ID 并覆盖历史记录。</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；original candidate adversarial P5 probe exit 1</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>接受并依赖 checksum；仅修 writer；在 domain validator 强制单调 sequence</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>TrainingQueue/ArmyRegistry validator 解析自身 ID namespace，并要求 next sequence 大于现有最大值；保留两条 adversarial regression。</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>修复阻断了 checksum 合法但领域内部倒退的快照；仍需不同 reviewer 独立接受。</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>中</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Persistence reviewer</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>V5-P2-T007,V5-P3-T006,V5-P5-T005</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>MITIGATED_PENDING_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
@@ -26868,7 +26906,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R493c139ecebc4c49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ad3451472ad4067"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27136,6 +27174,29 @@
       </x:c>
       <x:c r="G13"/>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>1.0.1-v5-g2-repair-001</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Independent repair reviewer</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>V5 G2 独立复审发现 stable-ID sequence 冷恢复缺陷并完成最小修复</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>TrainingQueue/ArmyRegistry validation、P5 adversarial tests、review/run/risk/baseline records；16 runtime tasks 保持 pending</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>修复 reviewer 不得自审接受；下一 Gate 仍是全新独立复审，不进入 G3/G4/V6</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -27143,7 +27204,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0beed921db3a40a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd977eed1ccb94d64"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27199,13 +27260,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="29" t="str">
-        <x:v>G2 runtime candidate 已实现但待独立复审；仍禁止 G3/G4/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
+        <x:v>G2 repair candidate 已形成但未获独立接受；仍禁止 G3/G4/G5/G6/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>G1 independently accepted；G2 P2/P3/P4/P5 与 automated vertical loop 已形成 candidate，但未获独立接受</x:v>
+        <x:v>原 candidate 的 stable-ID sequence validator 缺陷已修复；修复者不能签发独立通过</x:v>
       </x:c>
       <x:c r="D5" s="29" t="str">
-        <x:v>V5-G0/G1 VERIFIED；V5-G2 IMPLEMENTED_PENDING_REVIEW；后续门保持原状态</x:v>
+        <x:v>V5-G0/G1 VERIFIED；V5-G2 REPAIRED_PENDING_INDEPENDENT_REVIEW；后续门保持原状态</x:v>
       </x:c>
       <x:c r="E5" s="8" t="s">
         <x:v>1573</x:v>
@@ -27354,7 +27415,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8fe008c8056487a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra21f039da64e4f5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27778,13 +27839,13 @@
         <x:v>V6 只放宽 active policy，不更换集合容器</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>独立 G2 package review 尚未完成</x:v>
+        <x:v>stable-ID sequence guard 已修复；等待全新 independent reviewer 复验冷恢复后不复用 ID</x:v>
       </x:c>
       <x:c r="K13" s="9" t="s">
         <x:v>67</x:v>
       </x:c>
       <x:c r="L13" s="10" t="str">
-        <x:v>runtime 已实现/待独立复审</x:v>
+        <x:v>runtime repaired / pending fresh independent review</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" hidden="0" customHeight="1">
@@ -27816,13 +27877,13 @@
         <x:v>V1 三兼容字段只读迁入唯一 TrainingQueue</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>独立 G2 package review 尚未完成</x:v>
+        <x:v>stable-ID sequence guard 已修复；等待全新 independent reviewer 复验冷恢复后不复用 ID</x:v>
       </x:c>
       <x:c r="K14" s="9" t="s">
         <x:v>67</x:v>
       </x:c>
       <x:c r="L14" s="10" t="str">
-        <x:v>runtime 已实现/待独立复审</x:v>
+        <x:v>runtime repaired / pending fresh independent review</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="44" hidden="0" customHeight="1">
@@ -28188,7 +28249,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bd4d02c9484400b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbb431b2cdb4a16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28327,16 +28388,16 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>P2/P3/P4/P5 checkpoints + G2 vertical-loop candidate；exact 8 protected S1A.2 untracked</x:v>
+        <x:v>G2 repair candidate e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 untracked</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>git log/status + protected SHA-256</x:v>
+        <x:v>git log/status + protected SHA-256 + independent adversarial probe</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>G2 runtime 已实现但只为 IMPLEMENTED_PENDING_INDEPENDENT_REVIEW</x:v>
+        <x:v>原 cd7be2b 被独立复审发现 stable-ID sequence 单调性缺陷；已修复但不得由修复 reviewer 自行接受</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" hidden="0" customHeight="1">
@@ -28410,16 +28471,16 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>无持续 GUI PID；正式三场景 headless smoke 与 editor scan 为当前证据</x:v>
+        <x:v>无持续 GUI PID；正式 city/Blackstone/C0 与 editor scan 均 exit 0</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
       </x:c>
       <x:c r="E15" s="10" t="str">
-        <x:v>不把旧 PID 或历史 dirty 标题当当前运行身份</x:v>
+        <x:v>本轮只验证 headless runtime，不进入 G4 实际窗口门</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" hidden="0" customHeight="1">
@@ -28574,16 +28635,16 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>V5 SaveEnvelopeV1 + CampaignSnapshotV2 writer/migrator implemented</x:v>
+        <x:v>V5 SaveEnvelopeV1 + CampaignSnapshotV2 repair candidate</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>scripts/state/v5_campaign_* + TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md</x:v>
+        <x:v>scripts/state/v5_campaign_* + docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>S1A.2 八文件仅作为只读迁移输入与机制参考，仍非 V5 writer/schema</x:v>
+        <x:v>TrainingQueue/ArmyRegistry restore validator 已拒绝倒退 sequence；S1A.2 仍非 V5 writer/schema</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="38" hidden="0" customHeight="1">
@@ -28591,16 +28652,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>V5 focused 6/6 166；tracked 33/33 1720；all-present 35/35 1852 / 1886 PASS</x:v>
+        <x:v>V5 focused 6/6 168；tracked 33/33 1722；all-present 35/35 1854 / 1888 PASS</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
-        <x:v>all-present 含受保护 S1A.2 112 条与 V5 纵向闭环 20 条</x:v>
+        <x:v>相对原 candidate 各增加 2 条 sequence rollback adversarial assertions</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" hidden="0" customHeight="1">
@@ -28614,10 +28675,10 @@
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>/tmp/txwzs-v5-g2-full.M4M7T7 + final closeout commands</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>只把测试名中的 expected failure 文本当通过描述，不当错误签名</x:v>
+        <x:v>修复后全量回归；不构成修复 reviewer 自行接受</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" hidden="0" customHeight="1">
@@ -28625,16 +28686,16 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>023f11a P2；a95f510 P3；8a6e65a P4；ee32d84 P5；final G2 candidate this revision</x:v>
+        <x:v>023f11a P2；a95f510 P3；8a6e65a P4；ee32d84 P5；cd7be2b original candidate；e2c1096f858d571d4621b93174d3848406b42ffa repair</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>git log --oneline</x:v>
+        <x:v>git log --oneline + review report</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>各工作包均有可回滚本地 checkpoint；无 push</x:v>
+        <x:v>下一位 reviewer 必须绑定 repair checkpoint 并重验精确修改范围</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" hidden="0" customHeight="1">
@@ -28642,7 +28703,7 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>exact eight SHA-256 unchanged after G2 runtime and all-present regression</x:v>
+        <x:v>exact eight SHA-256 unchanged before/after review and repair regression</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
         <x:v>CONFIRMED</x:v>
@@ -28695,7 +28756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5296c92cee74496"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd77567f1adc4ecd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29320,7 +29381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc37537f8f2624072"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7454cfb5d33f4735"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -31464,16 +31525,18 @@
       </x:c>
       <x:c r="AD22" s="10"/>
       <x:c r="AE22" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF22" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF22" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG22" s="10"/>
       <x:c r="AH22" s="23" t="n">
         <x:f aca="0">IF(AND($Z22="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG22,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI22" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ22" s="9" t="s">
         <x:v>462</x:v>
@@ -31567,16 +31630,18 @@
       </x:c>
       <x:c r="AD23" s="10"/>
       <x:c r="AE23" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF23" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF23" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG23" s="10"/>
       <x:c r="AH23" s="23" t="n">
         <x:f aca="0">IF(AND($Z23="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG23,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI23" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ23" s="9" t="s">
         <x:v>462</x:v>
@@ -31777,16 +31842,18 @@
       </x:c>
       <x:c r="AD25" s="10"/>
       <x:c r="AE25" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF25" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF25" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG25" s="10"/>
       <x:c r="AH25" s="23" t="n">
         <x:f aca="0">IF(AND($Z25="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG25,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI25" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ25" s="9" t="s">
         <x:v>462</x:v>
@@ -31880,16 +31947,18 @@
       </x:c>
       <x:c r="AD26" s="10"/>
       <x:c r="AE26" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF26" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF26" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG26" s="10"/>
       <x:c r="AH26" s="23" t="n">
         <x:f aca="0">IF(AND($Z26="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG26,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI26" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ26" s="9" t="s">
         <x:v>462</x:v>
@@ -31983,16 +32052,18 @@
       </x:c>
       <x:c r="AD27" s="10"/>
       <x:c r="AE27" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF27" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF27" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG27" s="10"/>
       <x:c r="AH27" s="23" t="n">
         <x:f aca="0">IF(AND($Z27="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG27,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI27" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ27" s="9" t="s">
         <x:v>462</x:v>
@@ -32193,16 +32264,18 @@
       </x:c>
       <x:c r="AD29" s="10"/>
       <x:c r="AE29" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF29" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF29" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG29" s="10"/>
       <x:c r="AH29" s="23" t="n">
         <x:f aca="0">IF(AND($Z29="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG29,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI29" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ29" s="9" t="s">
         <x:v>462</x:v>
@@ -32296,16 +32369,18 @@
       </x:c>
       <x:c r="AD30" s="10"/>
       <x:c r="AE30" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF30" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF30" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG30" s="10"/>
       <x:c r="AH30" s="23" t="n">
         <x:f aca="0">IF(AND($Z30="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG30,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI30" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ30" s="9" t="s">
         <x:v>462</x:v>
@@ -32399,16 +32474,18 @@
       </x:c>
       <x:c r="AD31" s="10"/>
       <x:c r="AE31" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF31" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF31" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG31" s="10"/>
       <x:c r="AH31" s="23" t="n">
         <x:f aca="0">IF(AND($Z31="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG31,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI31" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ31" s="9" t="s">
         <x:v>462</x:v>
@@ -32502,16 +32579,18 @@
       </x:c>
       <x:c r="AD32" s="10"/>
       <x:c r="AE32" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF32" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF32" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG32" s="10"/>
       <x:c r="AH32" s="23" t="n">
         <x:f aca="0">IF(AND($Z32="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG32,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI32" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ32" s="9" t="s">
         <x:v>462</x:v>
@@ -32605,16 +32684,18 @@
       </x:c>
       <x:c r="AD33" s="10"/>
       <x:c r="AE33" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF33" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF33" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG33" s="10"/>
       <x:c r="AH33" s="23" t="n">
         <x:f aca="0">IF(AND($Z33="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG33,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI33" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ33" s="9" t="s">
         <x:v>462</x:v>
@@ -32815,16 +32896,18 @@
       </x:c>
       <x:c r="AD35" s="10"/>
       <x:c r="AE35" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF35" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF35" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG35" s="10"/>
       <x:c r="AH35" s="23" t="n">
         <x:f aca="0">IF(AND($Z35="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG35,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI35" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ35" s="9" t="s">
         <x:v>462</x:v>
@@ -32918,16 +33001,18 @@
       </x:c>
       <x:c r="AD36" s="10"/>
       <x:c r="AE36" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF36" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF36" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG36" s="10"/>
       <x:c r="AH36" s="23" t="n">
         <x:f aca="0">IF(AND($Z36="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG36,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI36" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ36" s="9" t="s">
         <x:v>462</x:v>
@@ -33021,16 +33106,18 @@
       </x:c>
       <x:c r="AD37" s="10"/>
       <x:c r="AE37" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF37" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF37" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG37" s="10"/>
       <x:c r="AH37" s="23" t="n">
         <x:f aca="0">IF(AND($Z37="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG37,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI37" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ37" s="9" t="s">
         <x:v>462</x:v>
@@ -33433,16 +33520,18 @@
       </x:c>
       <x:c r="AD41" s="10"/>
       <x:c r="AE41" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF41" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF41" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG41" s="10"/>
       <x:c r="AH41" s="23" t="n">
         <x:f aca="0">IF(AND($Z41="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG41,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI41" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ41" s="9" t="s">
         <x:v>462</x:v>
@@ -33536,16 +33625,18 @@
       </x:c>
       <x:c r="AD42" s="10"/>
       <x:c r="AE42" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF42" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF42" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG42" s="10"/>
       <x:c r="AH42" s="23" t="n">
         <x:f aca="0">IF(AND($Z42="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG42,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI42" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ42" s="9" t="s">
         <x:v>462</x:v>
@@ -33639,16 +33730,18 @@
       </x:c>
       <x:c r="AD43" s="10"/>
       <x:c r="AE43" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7</x:v>
-      </x:c>
-      <x:c r="AF43" s="10"/>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
+      <x:c r="AF43" s="10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
       <x:c r="AG43" s="10"/>
       <x:c r="AH43" s="23" t="n">
         <x:f aca="0">IF(AND($Z43="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG43,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI43" s="10" t="str">
-        <x:v>运行时与自动化证据已实现；等待不同 reviewer 独立复跑并裁决，不得自标 VERIFIED。</x:v>
+        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
       </x:c>
       <x:c r="AJ43" s="9" t="s">
         <x:v>462</x:v>
@@ -38314,7 +38407,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5d33579fa4346d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba09a6f80a4a4936"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38776,10 +38869,10 @@
       <x:c r="I14" s="10"/>
       <x:c r="J14" s="10"/>
       <x:c r="K14" s="10" t="str">
-        <x:v>Independent Codex at package gate</x:v>
+        <x:v>/root/v5_g2_independent_reviewer</x:v>
       </x:c>
       <x:c r="L14" s="19" t="str">
-        <x:v>V5-G2 runtime candidate implemented: P2/P3/P4/P5 + 20-assertion vertical loop; V5 focused 166; tracked 33/33 1720; all-present 35/35 1852 / 1886 PASS. Independent acceptance still required.</x:v>
+        <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW：原 candidate cd7be2b 接受倒退 TrainingQueue/ArmyRegistry sequence，恢复后可能复用 stable ID；已修复并通过 6/6 168、tracked 33/33 1722、all-present 35/35 1854/1888，但修复 reviewer 不得自审接受。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" hidden="0" customHeight="1">
@@ -40324,7 +40417,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6ba8aa97e33428d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a57a5702e504f95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40708,9 +40801,11 @@
         <x:v>1146</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J13" s="10"/>
+        <x:v>PASS_REPAIR_AGENT</x:v>
+      </x:c>
+      <x:c r="J13" s="10" t="str">
+        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+      </x:c>
       <x:c r="K13" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -40741,9 +40836,11 @@
         <x:v>1151</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J14" s="10"/>
+        <x:v>PASS_REPAIR_AGENT</x:v>
+      </x:c>
+      <x:c r="J14" s="10" t="str">
+        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+      </x:c>
       <x:c r="K14" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -40807,9 +40904,11 @@
         <x:v>1160</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J16" s="10"/>
+        <x:v>PASS_REPAIR_AGENT</x:v>
+      </x:c>
+      <x:c r="J16" s="10" t="str">
+        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+      </x:c>
       <x:c r="K16" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -40840,9 +40939,11 @@
         <x:v>1165</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J17" s="10"/>
+        <x:v>PASS_REPAIR_AGENT</x:v>
+      </x:c>
+      <x:c r="J17" s="10" t="str">
+        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+      </x:c>
       <x:c r="K17" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -40873,9 +40974,11 @@
         <x:v>1170</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J18" s="10"/>
+        <x:v>PASS_REPAIR_AGENT</x:v>
+      </x:c>
+      <x:c r="J18" s="10" t="str">
+        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+      </x:c>
       <x:c r="K18" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -41289,7 +41392,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbca9884ac5e146b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b3aed1779ac475c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41800,15 +41903,21 @@
       <x:c r="J13" s="9" t="s">
         <x:v>336</x:v>
       </x:c>
-      <x:c r="K13" s="9" t="s">
-        <x:v>1177</x:v>
-      </x:c>
-      <x:c r="L13" s="10"/>
+      <x:c r="K13" s="9" t="str">
+        <x:v>REPAIR_REQUIRED</x:v>
+      </x:c>
+      <x:c r="L13" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+      </x:c>
       <x:c r="M13" s="10" t="s">
         <x:v>1275</x:v>
       </x:c>
-      <x:c r="N13" s="25"/>
-      <x:c r="O13" s="10"/>
+      <x:c r="N13" s="25" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="O13" s="10" t="str">
+        <x:v>V5-G2</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="38" hidden="0" customHeight="1">
       <x:c r="A14" s="9" t="s">
@@ -42429,10 +42538,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K27" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L27" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M27" s="9" t="s">
         <x:v>314</x:v>
@@ -42474,10 +42583,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K28" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L28" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M28" s="9" t="s">
         <x:v>432</x:v>
@@ -42564,10 +42673,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K30" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L30" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M30" s="9" t="s">
         <x:v>432</x:v>
@@ -42609,10 +42718,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K31" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L31" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M31" s="9" t="s">
         <x:v>314</x:v>
@@ -42656,10 +42765,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K32" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L32" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M32" s="9" t="s">
         <x:v>314</x:v>
@@ -42746,10 +42855,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L34" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M34" s="9" t="s">
         <x:v>432</x:v>
@@ -42791,10 +42900,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K35" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L35" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M35" s="9" t="s">
         <x:v>432</x:v>
@@ -42836,10 +42945,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K36" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L36" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M36" s="9" t="s">
         <x:v>314</x:v>
@@ -42881,10 +42990,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K37" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L37" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M37" s="9" t="s">
         <x:v>432</x:v>
@@ -42928,10 +43037,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K38" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L38" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M38" s="9" t="s">
         <x:v>432</x:v>
@@ -43018,10 +43127,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K40" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L40" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M40" s="9" t="s">
         <x:v>432</x:v>
@@ -43063,10 +43172,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K41" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L41" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M41" s="9" t="s">
         <x:v>314</x:v>
@@ -43110,10 +43219,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K42" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L42" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M42" s="9" t="s">
         <x:v>432</x:v>
@@ -43286,10 +43395,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K46" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L46" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M46" s="9" t="s">
         <x:v>432</x:v>
@@ -43331,10 +43440,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K47" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L47" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M47" s="9" t="s">
         <x:v>432</x:v>
@@ -43378,10 +43487,10 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K48" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
+        <x:v>PASS_REPAIR_AGENT</x:v>
       </x:c>
       <x:c r="L48" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
       </x:c>
       <x:c r="M48" s="9" t="s">
         <x:v>432</x:v>
@@ -44454,7 +44563,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70f41f19128a4d4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8f4129fde74705"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44821,6 +44930,50 @@
       </x:c>
       <x:c r="N10" t="str">
         <x:v>Independent review required before V5-G2 VERIFIED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>RUN-V5-G2-INDEPENDENT-REVIEW-REPAIR-001</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>/root/v5_g2_independent_reviewer / GPT-5.6 Sol</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>V5-P2-T002,V5-P2-T003,V5-P2-T005,V5-P2-T006,V5-P2-T007,V5-P3-T002,V5-P3-T003,V5-P3-T004,V5-P3-T005,V5-P3-T006,V5-P4-T002,V5-P4-T003,V5-P4-T004,V5-P5-T003,V5-P5-T004,V5-P5-T005</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>cd7be2b4e65f453889c5f49a4922f788cca08a68；repair e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 U</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>TrainingQueue/ArmyRegistry validators；P5 smoke；review report；state/planning control</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Git/hash/40-file manifest；20 ownership checks；adversarial probe；focused/tracked/all-present；3 scenes/editor/diff；artifact-tool</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>original probe 2 FAIL；repair focused 6/6 168；tracked 33/33 1722；all-present 35/35 1854 / 1888 PASS；scenes/editor exit 0</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>修复 reviewer 不得接受自己的修复；G2 保持 pending；G3/G4/G5/G6/V6 未启动；S1A.2 保护不变</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 U</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>Fresh independent review of V5-G2 repair candidate</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>No；必须由不同 reviewer 复审后才可能验证 G2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -44853,7 +45006,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9abbad264e1b451f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red42bf0c10084aea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45174,6 +45327,50 @@
       </x:c>
       <x:c r="N9" t="str">
         <x:v>V5_G1_CONTRACT_PACKAGE_REVIEW_ACCEPTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>RVW-V5-G2-001</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>/root/v5_g2_independent_reviewer</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>V5-P2-T002,V5-P2-T003,V5-P2-T005,V5-P2-T006,V5-P2-T007,V5-P3-T002,V5-P3-T003,V5-P3-T004,V5-P3-T005,V5-P3-T006,V5-P4-T002,V5-P4-T003,V5-P4-T004,V5-P5-T003,V5-P5-T004,V5-P5-T005</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>reviewed cd7be2b4e65f453889c5f49a4922f788cca08a68；parent ee32d8445b11260a26501768da2c58abca78a113；repair e2c1096f858d571d4621b93174d3848406b42ffa；G2 chain 023f11a→a95f510→8a6e65a→ee32d84→cd7be2b；40 tracked files</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>stable IDs；single writers；conservation；idempotency；real BattleSession；V2 migration/generation/rollback/cold recovery；protected files</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>candidate probe exit 1 with 2 assertions；repair focused 6/6 168；tracked 33/33 1722；all-present 35/35 1854 / 1888；scenes/editor/diff 0</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>V2 validators accepted next_order_sequence/next_army_sequence lower than existing IDs, allowing ID reuse and historical record overwrite after restore</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>CRITICAL</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>P5 runner on original source: stale training and army sequence checks both FAIL；exit 1</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Validate generated ID namespace and require persisted next sequence greater than every existing sequence；retain adversarial regression</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>Minimal repair e2c1096f858d571d4621b93174d3848406b42ffa applied to TrainingQueue and ArmyRegistry validators；2 permanent assertions added；full regression passed</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>PENDING_FRESH_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -45206,7 +45403,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc30399e998f04aec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6103649bf962438e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: accept V5 G2 runtime package
</commit_message>
<xml_diff>
--- a/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
+++ b/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="Rf1ceb51e07ec4956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="R668369dab1b840e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="Ra64fa2bca96d4324"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="Rcaf24e6c79484f7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="R4a709ec37def4922"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="R58828281026940f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R3a07347bd81c486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="R423920dbf7954ca9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="R24f79f6a08234299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Ra16b2318e28f4718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="Re876932919c8454a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="Rb8e9cf8ee00448a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="R4a772bc04b564fc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="R7391969e41084ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="Re44e23596fc64c2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="R86d6408f8729478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="Rc8a0da75e2784bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="R116606fb9eab4494"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="Rbb372a5acb484e04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R4e8c644407bf4b6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="R601cb2873e984cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="Ra36cc5f6bd1f4e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R259fd6bcb8b64c1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="R4e166e3433374e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="R1f4dcedc2f684d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="R306db9c888004595"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25665,7 +25665,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>1.0.1-v5-g2-repair-001</x:v>
+        <x:v>1.0.2-v5-g2-fresh-review-accepted-003</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
         <x:v>6</x:v>
@@ -25684,7 +25684,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="D6" s="9" t="s">
         <x:v>10</x:v>
@@ -25705,7 +25705,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
+        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 VERIFIED；V5 IN_PROGRESS</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
         <x:v>13</x:v>
@@ -25724,7 +25724,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>由全新 reviewer 独立复审 V5-G2 repair candidate；复审前不得进入 G3/G4/G5/G6/V6</x:v>
+        <x:v>停止在 V5-G2 acceptance checkpoint；等待用户另行下令纯文档收敛；不得进入 G3/G4/G5/G6/V6</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
         <x:v>15</x:v>
@@ -25942,7 +25942,7 @@
       </x:c>
       <x:c r="F20" s="10" t="n">
         <x:f aca="0">COUNTIFS('03_任务总表'!$C$5:$C$200,D20,'03_任务总表'!$Z$5:$Z$200,"VERIFIED")</x:f>
-        <x:v>17</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G20" s="10" t="n">
         <x:f aca="0">COUNTIFS('03_任务总表'!$C$5:$C$200,D20,'03_任务总表'!$Z$5:$Z$200,"CANCELLED")</x:f>
@@ -25950,7 +25950,7 @@
       </x:c>
       <x:c r="H20" s="16" t="n">
         <x:f aca="0">IFERROR(F20/SUMIFS('03_任务总表'!$AH$5:$AH$200,'03_任务总表'!$C$5:$C$200,D20),0)</x:f>
-        <x:v>0.38636363636363635</x:v>
+        <x:v>0.75</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0">
@@ -25959,7 +25959,7 @@
       </x:c>
       <x:c r="B21" s="10" t="n">
         <x:f aca="0">COUNTIF('03_任务总表'!$Z$5:$Z$200,"IMPLEMENTED_PENDING_REVIEW")</x:f>
-        <x:v>16</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D21" s="9" t="s">
         <x:v>51</x:v>
@@ -26849,16 +26849,16 @@
         <x:v>V2 aggregate validator 若只检查 next sequence 为正而不高于既有 stable ID，冷恢复后的新训练/派遣会复用 ID 并覆盖历史记录。</x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；original candidate adversarial P5 probe exit 1</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；fab962c0a84024e7034c32e9d5c39debc1659c5f；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md；fresh probe 29/29</x:v>
       </x:c>
       <x:c r="E20" t="str">
         <x:v>接受并依赖 checksum；仅修 writer；在 domain validator 强制单调 sequence</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>TrainingQueue/ArmyRegistry validator 解析自身 ID namespace，并要求 next sequence 大于现有最大值；保留两条 adversarial regression。</x:v>
+        <x:v>TrainingQueue/ArmyRegistry validator 严格拒绝错误类型、范围、回退与 exhausted successor；Army 创建在 reservation/transaction/garrison 写入前失败。</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>修复阻断了 checksum 合法但领域内部倒退的快照；仍需不同 reviewer 独立接受。</x:v>
+        <x:v>fresh independent review 关闭该 G2 阻断；永久 adversarial regression 保留。G3 及后续 Gate 仍需各自验收。</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>中</x:v>
@@ -26873,7 +26873,7 @@
         <x:v>V5-P2-T007,V5-P3-T006,V5-P5-T005</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>MITIGATED_PENDING_INDEPENDENT_REVIEW</x:v>
+        <x:v>MITIGATED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -26906,7 +26906,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ad3451472ad4067"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd82df2c756543d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27197,6 +27197,29 @@
         <x:v>RVW-V5-G2-001</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>1.0.2-v5-g2-fresh-review-accepted-003</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Independent + Main Codex</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>fresh independent review 接受 V5-G2 stable-ID boundary repair</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>精确16项 runtime tasks→VERIFIED；V5-G2→VERIFIED；Review/Run/Risk/Baseline/主控镜像同步</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>完整提交链、四文件 diff、29/29 边界探针、51/51 P5、三组全量回归与 S1A.2 哈希均独立成立；停止在 G2</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>RVW-V5-G2-003</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -27204,7 +27227,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd977eed1ccb94d64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc99720aecd904f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27260,13 +27283,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="29" t="str">
-        <x:v>G2 repair candidate 已形成但未获独立接受；仍禁止 G3/G4/G5/G6/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
+        <x:v>V5-G2 已 fresh independently accepted；仍禁止 G3/G4/G5/G6/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>原 candidate 的 stable-ID sequence validator 缺陷已修复；修复者不能签发独立通过</x:v>
+        <x:v>stable-ID boundary repair 已由不同 reviewer 绑定完整提交链并独立通过；本轮只形成 acceptance checkpoint</x:v>
       </x:c>
       <x:c r="D5" s="29" t="str">
-        <x:v>V5-G0/G1 VERIFIED；V5-G2 REPAIRED_PENDING_INDEPENDENT_REVIEW；后续门保持原状态</x:v>
+        <x:v>V5-G0/G1/G2 VERIFIED；精确 16 项 runtime tasks VERIFIED；后续门保持 NOT_STARTED</x:v>
       </x:c>
       <x:c r="E5" s="8" t="s">
         <x:v>1573</x:v>
@@ -27415,7 +27438,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra21f039da64e4f5d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9cbd73025854e69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27839,13 +27862,13 @@
         <x:v>V6 只放宽 active policy，不更换集合容器</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>stable-ID sequence guard 已修复；等待全新 independent reviewer 复验冷恢复后不复用 ID</x:v>
-      </x:c>
-      <x:c r="K13" s="9" t="s">
-        <x:v>67</x:v>
+        <x:v>stable-ID sequence type/range/successor/exhaustion 与 pre-reservation failure 已由 fresh reviewer 独立接受</x:v>
+      </x:c>
+      <x:c r="K13" s="9" t="str">
+        <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="L13" s="10" t="str">
-        <x:v>runtime repaired / pending fresh independent review</x:v>
+        <x:v>runtime implemented / V5-G2 independently accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="44" hidden="0" customHeight="1">
@@ -27877,13 +27900,13 @@
         <x:v>V1 三兼容字段只读迁入唯一 TrainingQueue</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>stable-ID sequence guard 已修复；等待全新 independent reviewer 复验冷恢复后不复用 ID</x:v>
-      </x:c>
-      <x:c r="K14" s="9" t="s">
-        <x:v>67</x:v>
+        <x:v>stable-ID sequence type/range/successor/exhaustion 与合法 V1 空队列历史迁移已由 fresh reviewer 独立接受</x:v>
+      </x:c>
+      <x:c r="K14" s="9" t="str">
+        <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="L14" s="10" t="str">
-        <x:v>runtime repaired / pending fresh independent review</x:v>
+        <x:v>runtime implemented / V5-G2 independently accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="44" hidden="0" customHeight="1">
@@ -28181,13 +28204,13 @@
         <x:v>V1 read-only migration implemented；future versions reject</x:v>
       </x:c>
       <x:c r="J22" s="10" t="str">
-        <x:v>独立 G2 package review 尚未完成</x:v>
+        <x:v>V1→V2、codec/store/generation/fallback/cold restore 与 zero-partial-write 已由 fresh reviewer 独立接受</x:v>
       </x:c>
       <x:c r="K22" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="L22" s="10" t="str">
-        <x:v>runtime 已实现/待独立复审</x:v>
+        <x:v>runtime implemented / V5-G2 independently accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="44" hidden="0" customHeight="1">
@@ -28219,13 +28242,13 @@
         <x:v>无需第二 resolver；继续沿用 coordinator-bound authority</x:v>
       </x:c>
       <x:c r="J23" s="10" t="str">
-        <x:v>独立 G2 package review 尚未完成</x:v>
-      </x:c>
-      <x:c r="K23" s="9" t="s">
-        <x:v>67</x:v>
+        <x:v>真实 BattleSession facts、coordinator-bound Army settlement 与幂等 writeback 已由 fresh reviewer 独立接受</x:v>
+      </x:c>
+      <x:c r="K23" s="9" t="str">
+        <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="L23" s="10" t="str">
-        <x:v>Army writeback runtime 已实现/待独立复审</x:v>
+        <x:v>Army writeback runtime implemented / V5-G2 independently accepted</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28249,7 +28272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bbb431b2cdb4a16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0f644fea1cb4a5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28388,16 +28411,16 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>G2 repair candidate e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 untracked</x:v>
+        <x:v>G2 fresh independent review baseline 4d0fbfc5aefe07509db115f8f4f68e22aeda8a98；exact 8 protected S1A.2 untracked</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>git log/status + protected SHA-256 + independent adversarial probe</x:v>
+        <x:v>git log/status + docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md + protected SHA-256</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>原 cd7be2b 被独立复审发现 stable-ID sequence 单调性缺陷；已修复但不得由修复 reviewer 自行接受</x:v>
+        <x:v>fresh reviewer 绑定完整提交链与四文件 repair，V5-G2 已独立接受；不释放 G3</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" hidden="0" customHeight="1">
@@ -28635,16 +28658,16 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>V5 SaveEnvelopeV1 + CampaignSnapshotV2 repair candidate</x:v>
+        <x:v>V5 SaveEnvelopeV1 + CampaignSnapshotV2；V5-G2 runtime package independently accepted</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>scripts/state/v5_campaign_* + docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>scripts/state/v5_campaign_* + docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>TrainingQueue/ArmyRegistry restore validator 已拒绝倒退 sequence；S1A.2 仍非 V5 writer/schema</x:v>
+        <x:v>stable-ID sequence、V1→V2、zero-partial-write、disk/codec/store/cold restore/fallback 边界独立通过</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="38" hidden="0" customHeight="1">
@@ -28652,16 +28675,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>V5 focused 6/6 168；tracked 33/33 1722；all-present 35/35 1854 / 1888 PASS</x:v>
+        <x:v>V5 focused 6/6 185；tracked 33/33 1739；all-present 35/35 1871 assertions / 1905 PASS</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="E26" s="10" t="str">
-        <x:v>相对原 candidate 各增加 2 条 sequence rollback adversarial assertions</x:v>
+        <x:v>fresh review 相对 repair reviewer 基线新增永久 stable-ID/domain/cold-boundary coverage；runner 数无差异</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" hidden="0" customHeight="1">
@@ -28669,16 +28692,16 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>PASS / exit 0；formal city/Blackstone/C0 exits 0；final error signatures 0</x:v>
+        <x:v>PASS / exit 0；formal city/Blackstone/C0 与 editor scan exit 0；final error signatures 0</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>修复后全量回归；不构成修复 reviewer 自行接受</x:v>
+        <x:v>fresh reviewer 独立重跑；不构成 G3、实际窗口或用户试玩验收</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" hidden="0" customHeight="1">
@@ -28686,16 +28709,16 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>023f11a P2；a95f510 P3；8a6e65a P4；ee32d84 P5；cd7be2b original candidate；e2c1096f858d571d4621b93174d3848406b42ffa repair</x:v>
+        <x:v>cd7be2b4e65f453889c5f49a4922f788cca08a68 → e2c1096f858d571d4621b93174d3848406b42ffa → 5d659243 → fab962c0a84024e7034c32e9d5c39debc1659c5f → 4d0fbfc5aefe07509db115f8f4f68e22aeda8a98</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
-        <x:v>git log --oneline + review report</x:v>
+        <x:v>git merge-base --is-ancestor + git show + four-file repair diff</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>下一位 reviewer 必须绑定 repair checkpoint 并重验精确修改范围</x:v>
+        <x:v>4d0fbfc 为现场文档 checkpoint；acceptance checkpoint 仅含报告、状态和主控同步</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" hidden="0" customHeight="1">
@@ -28703,16 +28726,16 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>exact eight SHA-256 unchanged before/after review and repair regression</x:v>
+        <x:v>exact eight SHA-256 unchanged before/after fresh review and planning sync</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
         <x:v>CONFIRMED</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>shasum -a 256 + git status + staged exclusion</x:v>
+        <x:v>shasum -a 256 + git status + docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="E29" s="10" t="str">
-        <x:v>八文件未修改、未暂存、未提交</x:v>
+        <x:v>八文件保持唯一 untracked、unstaged；不属于本 acceptance checkpoint</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="38" hidden="0" customHeight="1">
@@ -28756,7 +28779,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd77567f1adc4ecd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96bf1ab7aa034965"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28971,7 +28994,7 @@
       </x:c>
       <x:c r="P6" s="16" t="n">
         <x:f aca="0">IFERROR(COUNTIFS('03_任务总表'!$C$5:$C$200,$A6,'03_任务总表'!$Z$5:$Z$200,"VERIFIED")/SUMIFS('03_任务总表'!$AH$5:$AH$200,'03_任务总表'!$C$5:$C$200,$A6),0)</x:f>
-        <x:v>0.38636363636363635</x:v>
+        <x:v>0.75</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="44" hidden="0" customHeight="1">
@@ -29381,7 +29404,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7454cfb5d33f4735"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re404080757b64b72"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -31514,7 +31537,7 @@
         <x:v>314</x:v>
       </x:c>
       <x:c r="Z22" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA22" s="10"/>
       <x:c r="AB22" s="10" t="str">
@@ -31523,12 +31546,14 @@
       <x:c r="AC22" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD22" s="10"/>
+      <x:c r="AD22" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE22" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF22" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG22" s="10"/>
       <x:c r="AH22" s="23" t="n">
@@ -31536,7 +31561,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI22" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ22" s="9" t="s">
         <x:v>462</x:v>
@@ -31619,7 +31644,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z23" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA23" s="10"/>
       <x:c r="AB23" s="10" t="str">
@@ -31628,12 +31653,14 @@
       <x:c r="AC23" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD23" s="10"/>
+      <x:c r="AD23" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE23" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF23" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG23" s="10"/>
       <x:c r="AH23" s="23" t="n">
@@ -31641,7 +31668,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI23" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ23" s="9" t="s">
         <x:v>462</x:v>
@@ -31831,7 +31858,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z25" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA25" s="10"/>
       <x:c r="AB25" s="10" t="str">
@@ -31840,12 +31867,14 @@
       <x:c r="AC25" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD25" s="10"/>
+      <x:c r="AD25" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE25" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF25" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG25" s="10"/>
       <x:c r="AH25" s="23" t="n">
@@ -31853,7 +31882,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI25" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ25" s="9" t="s">
         <x:v>462</x:v>
@@ -31936,7 +31965,7 @@
         <x:v>314</x:v>
       </x:c>
       <x:c r="Z26" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA26" s="10"/>
       <x:c r="AB26" s="10" t="str">
@@ -31945,12 +31974,14 @@
       <x:c r="AC26" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD26" s="10"/>
+      <x:c r="AD26" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE26" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF26" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG26" s="10"/>
       <x:c r="AH26" s="23" t="n">
@@ -31958,7 +31989,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI26" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ26" s="9" t="s">
         <x:v>462</x:v>
@@ -32041,7 +32072,7 @@
         <x:v>314</x:v>
       </x:c>
       <x:c r="Z27" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA27" s="10"/>
       <x:c r="AB27" s="10" t="str">
@@ -32050,12 +32081,14 @@
       <x:c r="AC27" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD27" s="10"/>
+      <x:c r="AD27" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE27" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF27" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG27" s="10"/>
       <x:c r="AH27" s="23" t="n">
@@ -32063,7 +32096,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI27" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ27" s="9" t="s">
         <x:v>462</x:v>
@@ -32253,7 +32286,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z29" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA29" s="10"/>
       <x:c r="AB29" s="10" t="str">
@@ -32262,12 +32295,14 @@
       <x:c r="AC29" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD29" s="10"/>
+      <x:c r="AD29" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE29" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF29" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG29" s="10"/>
       <x:c r="AH29" s="23" t="n">
@@ -32275,7 +32310,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI29" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ29" s="9" t="s">
         <x:v>462</x:v>
@@ -32358,7 +32393,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z30" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA30" s="10"/>
       <x:c r="AB30" s="10" t="str">
@@ -32367,12 +32402,14 @@
       <x:c r="AC30" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD30" s="10"/>
+      <x:c r="AD30" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE30" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF30" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG30" s="10"/>
       <x:c r="AH30" s="23" t="n">
@@ -32380,7 +32417,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI30" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ30" s="9" t="s">
         <x:v>462</x:v>
@@ -32463,7 +32500,7 @@
         <x:v>314</x:v>
       </x:c>
       <x:c r="Z31" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA31" s="10"/>
       <x:c r="AB31" s="10" t="str">
@@ -32472,12 +32509,14 @@
       <x:c r="AC31" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD31" s="10"/>
+      <x:c r="AD31" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE31" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF31" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG31" s="10"/>
       <x:c r="AH31" s="23" t="n">
@@ -32485,7 +32524,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI31" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ31" s="9" t="s">
         <x:v>462</x:v>
@@ -32568,7 +32607,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z32" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA32" s="10"/>
       <x:c r="AB32" s="10" t="str">
@@ -32577,12 +32616,14 @@
       <x:c r="AC32" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD32" s="10"/>
+      <x:c r="AD32" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE32" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF32" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG32" s="10"/>
       <x:c r="AH32" s="23" t="n">
@@ -32590,7 +32631,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI32" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ32" s="9" t="s">
         <x:v>462</x:v>
@@ -32673,7 +32714,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z33" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA33" s="10"/>
       <x:c r="AB33" s="10" t="str">
@@ -32682,12 +32723,14 @@
       <x:c r="AC33" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD33" s="10"/>
+      <x:c r="AD33" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE33" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF33" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG33" s="10"/>
       <x:c r="AH33" s="23" t="n">
@@ -32695,7 +32738,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI33" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ33" s="9" t="s">
         <x:v>462</x:v>
@@ -32885,7 +32928,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z35" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA35" s="10"/>
       <x:c r="AB35" s="10" t="str">
@@ -32894,12 +32937,14 @@
       <x:c r="AC35" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD35" s="10"/>
+      <x:c r="AD35" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE35" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF35" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG35" s="10"/>
       <x:c r="AH35" s="23" t="n">
@@ -32907,7 +32952,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI35" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ35" s="9" t="s">
         <x:v>462</x:v>
@@ -32990,7 +33035,7 @@
         <x:v>314</x:v>
       </x:c>
       <x:c r="Z36" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA36" s="10"/>
       <x:c r="AB36" s="10" t="str">
@@ -32999,12 +33044,14 @@
       <x:c r="AC36" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD36" s="10"/>
+      <x:c r="AD36" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE36" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF36" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG36" s="10"/>
       <x:c r="AH36" s="23" t="n">
@@ -33012,7 +33059,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI36" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ36" s="9" t="s">
         <x:v>462</x:v>
@@ -33095,7 +33142,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z37" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA37" s="10"/>
       <x:c r="AB37" s="10" t="str">
@@ -33104,12 +33151,14 @@
       <x:c r="AC37" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD37" s="10"/>
+      <x:c r="AD37" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE37" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF37" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG37" s="10"/>
       <x:c r="AH37" s="23" t="n">
@@ -33117,7 +33166,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI37" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ37" s="9" t="s">
         <x:v>462</x:v>
@@ -33509,7 +33558,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z41" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA41" s="10"/>
       <x:c r="AB41" s="10" t="str">
@@ -33518,12 +33567,14 @@
       <x:c r="AC41" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD41" s="10"/>
+      <x:c r="AD41" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE41" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF41" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG41" s="10"/>
       <x:c r="AH41" s="23" t="n">
@@ -33531,7 +33582,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI41" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ41" s="9" t="s">
         <x:v>462</x:v>
@@ -33614,7 +33665,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z42" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA42" s="10"/>
       <x:c r="AB42" s="10" t="str">
@@ -33623,12 +33674,14 @@
       <x:c r="AC42" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD42" s="10"/>
+      <x:c r="AD42" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE42" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF42" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG42" s="10"/>
       <x:c r="AH42" s="23" t="n">
@@ -33636,7 +33689,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI42" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ42" s="9" t="s">
         <x:v>462</x:v>
@@ -33719,7 +33772,7 @@
         <x:v>432</x:v>
       </x:c>
       <x:c r="Z43" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA43" s="10"/>
       <x:c r="AB43" s="10" t="str">
@@ -33728,12 +33781,14 @@
       <x:c r="AC43" s="10" t="str">
         <x:v>2026-07-30</x:v>
       </x:c>
-      <x:c r="AD43" s="10"/>
+      <x:c r="AD43" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
       <x:c r="AE43" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_001.md；/tmp/txwzs-v5-g2-full.M4M7T7；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="AF43" s="10" t="str">
-        <x:v>RVW-V5-G2-001</x:v>
+        <x:v>RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="AG43" s="10"/>
       <x:c r="AH43" s="23" t="n">
@@ -33741,7 +33796,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AI43" s="10" t="str">
-        <x:v>独立复审发现 V2 接受倒退 stable-ID sequence；原子修复 e2c1096f858d571d4621b93174d3848406b42ffa 已全量回归。状态保持 IMPLEMENTED_PENDING_REVIEW，必须由全新 reviewer 重验。</x:v>
+        <x:v>RVW-V5-G2-001 发现 stable-ID sequence 缺陷；fab962c 完成四文件最小修复与永久回归。RVW-V5-G2-003 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc，独立通过 29/29 边界探针、P5 51/51、focused 6/6·185、tracked 33/33·1739、all-present 35/35·1871/1905；本任务仅在 V5-G2 VERIFIED，G3 及以后未启动。</x:v>
       </x:c>
       <x:c r="AJ43" s="9" t="s">
         <x:v>462</x:v>
@@ -38407,7 +38462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba09a6f80a4a4936"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0c8d7935fa7488a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38864,15 +38919,19 @@
         <x:v>986</x:v>
       </x:c>
       <x:c r="H14" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
-      </x:c>
-      <x:c r="I14" s="10"/>
-      <x:c r="J14" s="10"/>
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="I14" s="10" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+      <x:c r="J14" s="10" t="str">
+        <x:v>Independent Codex</x:v>
+      </x:c>
       <x:c r="K14" s="10" t="str">
-        <x:v>/root/v5_g2_independent_reviewer</x:v>
+        <x:v>/root/v5_g2_boundary_fresh_independent_reviewer_003</x:v>
       </x:c>
       <x:c r="L14" s="19" t="str">
-        <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW：原 candidate cd7be2b 接受倒退 TrainingQueue/ArmyRegistry sequence，恢复后可能复用 stable ID；已修复并通过 6/6 168、tracked 33/33 1722、all-present 35/35 1854/1888，但修复 reviewer 不得自审接受。</x:v>
+        <x:v>V5_G2_RUNTIME_PACKAGE_REVIEW_ACCEPTED：fresh reviewer 绑定 cd7be2b→e2c1096→5d659243→fab962c→4d0fbfc；四文件 repair；independent probe 29/29；P5 51/51；focused 6/6·185；tracked 33/33·1739；all-present 35/35·1871/1905；S1A.2 八文件不变。只接受 G2，G3–G6/V6 保持 NOT_STARTED。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" hidden="0" customHeight="1">
@@ -40417,7 +40476,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a57a5702e504f95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85a75b0531de4bc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40669,11 +40728,13 @@
         <x:v>1124</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J9" s="10"/>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J9" s="10" t="str">
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
+      </x:c>
       <x:c r="K9" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" hidden="0" customHeight="1">
@@ -40702,11 +40763,13 @@
         <x:v>1130</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J10" s="10"/>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J10" s="10" t="str">
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
+      </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" hidden="0" customHeight="1">
@@ -40735,11 +40798,13 @@
         <x:v>1135</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J11" s="10"/>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J11" s="10" t="str">
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
+      </x:c>
       <x:c r="K11" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" hidden="0" customHeight="1">
@@ -40768,9 +40833,11 @@
         <x:v>1141</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J12" s="10"/>
+        <x:v>PASS_G2_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J12" s="10" t="str">
+        <x:v>G2_RUNTIME_ACCEPTED / RVW-V5-G2-003；V5-P6-T003 尚未启动</x:v>
+      </x:c>
       <x:c r="K12" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
       </x:c>
@@ -40801,13 +40868,13 @@
         <x:v>1146</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="J13" s="10" t="str">
-        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="K13" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="38" hidden="0" customHeight="1">
@@ -40836,13 +40903,13 @@
         <x:v>1151</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="J14" s="10" t="str">
-        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="K14" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" hidden="0" customHeight="1">
@@ -40871,11 +40938,13 @@
         <x:v>1156</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
-        <x:v>PASS_MAIN_AGENT</x:v>
-      </x:c>
-      <x:c r="J15" s="10"/>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+      <x:c r="J15" s="10" t="str">
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
+      </x:c>
       <x:c r="K15" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" hidden="0" customHeight="1">
@@ -40904,13 +40973,13 @@
         <x:v>1160</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="J16" s="10" t="str">
-        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="K16" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="38" hidden="0" customHeight="1">
@@ -40939,10 +41008,10 @@
         <x:v>1165</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_G2_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="J17" s="10" t="str">
-        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+        <x:v>G2_PERSISTENCE_ACCEPTED / RVW-V5-G2-003；V5-P7-T004 实际窗口重载尚未启动</x:v>
       </x:c>
       <x:c r="K17" s="9" t="str">
         <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
@@ -40974,13 +41043,13 @@
         <x:v>1170</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="J18" s="10" t="str">
-        <x:v>REPAIR_REQUIRED；修复完成，等待全新独立复审</x:v>
+        <x:v>ACCEPTED / RVW-V5-G2-003</x:v>
       </x:c>
       <x:c r="K18" s="9" t="str">
-        <x:v>IMPLEMENTED_PENDING_REVIEW</x:v>
+        <x:v>VERIFIED</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" hidden="0" customHeight="1">
@@ -41392,7 +41461,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b3aed1779ac475c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf86a71fdb81c4f63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41904,16 +41973,16 @@
         <x:v>336</x:v>
       </x:c>
       <x:c r="K13" s="9" t="str">
-        <x:v>REPAIR_REQUIRED</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L13" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md</x:v>
+        <x:v>docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M13" s="10" t="s">
         <x:v>1275</x:v>
       </x:c>
       <x:c r="N13" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O13" s="10" t="str">
         <x:v>V5-G2</x:v>
@@ -42538,16 +42607,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K27" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L27" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M27" s="9" t="s">
         <x:v>314</x:v>
       </x:c>
       <x:c r="N27" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O27" s="9" t="s">
         <x:v>462</x:v>
@@ -42583,16 +42652,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K28" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L28" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M28" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N28" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O28" s="9" t="s">
         <x:v>462</x:v>
@@ -42673,16 +42742,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K30" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L30" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M30" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N30" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O30" s="9" t="s">
         <x:v>462</x:v>
@@ -42718,16 +42787,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K31" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L31" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M31" s="9" t="s">
         <x:v>314</x:v>
       </x:c>
       <x:c r="N31" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O31" s="9" t="s">
         <x:v>462</x:v>
@@ -42765,16 +42834,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K32" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L32" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P2_TRAINING_TIME_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_training_queue_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M32" s="9" t="s">
         <x:v>314</x:v>
       </x:c>
       <x:c r="N32" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O32" s="9" t="s">
         <x:v>462</x:v>
@@ -42855,16 +42924,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L34" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M34" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N34" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O34" s="9" t="s">
         <x:v>462</x:v>
@@ -42900,16 +42969,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K35" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L35" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M35" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N35" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O35" s="9" t="s">
         <x:v>462</x:v>
@@ -42945,16 +43014,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K36" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L36" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M36" s="9" t="s">
         <x:v>314</x:v>
       </x:c>
       <x:c r="N36" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O36" s="9" t="s">
         <x:v>462</x:v>
@@ -42990,16 +43059,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K37" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L37" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M37" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N37" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O37" s="9" t="s">
         <x:v>462</x:v>
@@ -43037,16 +43106,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K38" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L38" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P3_ARMY_STATE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_army_state_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M38" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N38" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O38" s="9" t="s">
         <x:v>462</x:v>
@@ -43127,16 +43196,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K40" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L40" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M40" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N40" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O40" s="9" t="s">
         <x:v>462</x:v>
@@ -43172,16 +43241,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K41" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L41" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M41" s="9" t="s">
         <x:v>314</x:v>
       </x:c>
       <x:c r="N41" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O41" s="9" t="s">
         <x:v>462</x:v>
@@ -43219,16 +43288,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K42" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L42" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P4_ENCOUNTER_WRITEBACK_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_encounter_writeback_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M42" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N42" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O42" s="9" t="s">
         <x:v>462</x:v>
@@ -43395,16 +43464,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K46" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L46" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M46" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N46" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O46" s="9" t="s">
         <x:v>462</x:v>
@@ -43440,16 +43509,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K47" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L47" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M47" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N47" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O47" s="9" t="s">
         <x:v>462</x:v>
@@ -43487,16 +43556,16 @@
         <x:v>1321</x:v>
       </x:c>
       <x:c r="K48" s="9" t="str">
-        <x:v>PASS_REPAIR_AGENT</x:v>
+        <x:v>PASS_INDEPENDENT_REVIEW</x:v>
       </x:c>
       <x:c r="L48" s="10" t="str">
-        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>docs/reports/TXWZS_V5_P5_CAMPAIGN_PERSISTENCE_IMPLEMENTATION_001.md；/tmp/txwzs-v5-g2-full.M4M7T7/all-present-run_v5_campaign_persistence_smoke.log；docs/reports/TXWZS_V5_G2_RUNTIME_PACKAGE_INDEPENDENT_REVIEW_001.md；repair e2c1096f858d571d4621b93174d3848406b42ffa；docs/reports/TXWZS_V5_G2_STABLE_ID_BOUNDARY_REPAIR_FRESH_INDEPENDENT_REVIEW_003.md</x:v>
       </x:c>
       <x:c r="M48" s="9" t="s">
         <x:v>432</x:v>
       </x:c>
       <x:c r="N48" s="25" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="O48" s="9" t="s">
         <x:v>462</x:v>
@@ -44563,7 +44632,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8f4129fde74705"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4db46b3cc5d4dd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44934,46 +45003,46 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>RUN-V5-G2-INDEPENDENT-REVIEW-REPAIR-001</x:v>
+        <x:v>RUN-V5-G2-FRESH-INDEPENDENT-REVIEW-003</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>2026-07-30</x:v>
+        <x:v>2026-07-31</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>/root/v5_g2_independent_reviewer / GPT-5.6 Sol</x:v>
+        <x:v>/root/v5_g2_boundary_fresh_independent_reviewer_003 / GPT-5.6 Sol high</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>V5-P2-T002,V5-P2-T003,V5-P2-T005,V5-P2-T006,V5-P2-T007,V5-P3-T002,V5-P3-T003,V5-P3-T004,V5-P3-T005,V5-P3-T006,V5-P4-T002,V5-P4-T003,V5-P4-T004,V5-P5-T003,V5-P5-T004,V5-P5-T005</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>cd7be2b4e65f453889c5f49a4922f788cca08a68；repair e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 U</x:v>
+        <x:v>4d0fbfc5aefe07509db115f8f4f68e22aeda8a98；exact 8 protected S1A.2 U；index empty</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>TrainingQueue/ArmyRegistry validators；P5 smoke；review report；state/planning control</x:v>
+        <x:v>Review 003 + CURRENT_STATE + planning workbook/MD/CSV synchronization only</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>Git/hash/40-file manifest；20 ownership checks；adversarial probe；focused/tracked/all-present；3 scenes/editor/diff；artifact-tool</x:v>
+        <x:v>commit-chain/ancestor/index/hash/four-file diff；fresh adversarial probe；focused/tracked/all-present；cold A/B/C；formal scenes/editor/diff/error；13-sheet workbook audit</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>original probe 2 FAIL；repair focused 6/6 168；tracked 33/33 1722；all-present 35/35 1854 / 1888 PASS；scenes/editor exit 0</x:v>
+        <x:v>probe 29/29；P5 51/51；focused 6/6 185；tracked 33/33 1739；all-present 35/35 1871 assertions / 1905 PASS；cold A/B/C 0/0/0</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
+        <x:v>V5_G2_RUNTIME_PACKAGE_REVIEW_ACCEPTED</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>修复 reviewer 不得接受自己的修复；G2 保持 pending；G3/G4/G5/G6/V6 未启动；S1A.2 保护不变</x:v>
+        <x:v>Accepts exact 16 runtime tasks and V5-G2 only；no P4-T005/P6/P7/G3-G6/V6；no source changes；S1A.2 protected</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>e2c1096f858d571d4621b93174d3848406b42ffa；exact 8 protected S1A.2 U</x:v>
+        <x:v>local acceptance checkpoint；exact 8 protected S1A.2 U</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>e2c1096f858d571d4621b93174d3848406b42ffa</x:v>
+        <x:v>acceptance checkpoint containing this planning revision</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>Fresh independent review of V5-G2 repair candidate</x:v>
+        <x:v>Stop before G3；await separately authorized Markdown convergence</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>No；必须由不同 reviewer 复审后才可能验证 G2</x:v>
+        <x:v>No；do not enter G3/push/deploy</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -45006,7 +45075,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red42bf0c10084aea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa4d04ce0e214c7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45371,6 +45440,50 @@
       </x:c>
       <x:c r="N10" t="str">
         <x:v>V5_G2_REPAIRED_PENDING_INDEPENDENT_REVIEW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>RVW-V5-G2-003</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>/root/v5_g2_boundary_fresh_independent_reviewer_003</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>V5-P2-T002,V5-P2-T003,V5-P2-T005,V5-P2-T006,V5-P2-T007,V5-P3-T002,V5-P3-T003,V5-P3-T004,V5-P3-T005,V5-P3-T006,V5-P4-T002,V5-P4-T003,V5-P4-T004,V5-P5-T003,V5-P5-T004,V5-P5-T005</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>cd7be2b4e65f453889c5f49a4922f788cca08a68 → e2c1096f858d571d4621b93174d3848406b42ffa → 5d659243 → fab962c0a84024e7034c32e9d5c39debc1659c5f → 4d0fbfc5aefe07509db115f8f4f68e22aeda8a98；repair diff exact 4 files</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>stable-ID domain/type/range/exhaustion；reservation-before-failure；V1→V2 historical day；zero partial writes；disk/codec/store/cold/fallback；protected hashes</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>fresh probe 29/29；P5 51/51；focused 6/6·185；tracked 33/33·1739；all-present 35/35·1871/1905；cold A/B/C 0/0/0；scenes/editor/diff/error 0</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>No new substantive defect</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>NONE</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>fresh independent checkout-bound review; temporary probe removed after permanent coverage was confirmed</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>Accept exact G2 runtime boundary and stop before G3</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>fab962c four-file repair retained; no review-time source change</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>ACCEPTED；candidate chain, assertions, hashes and protected state matched</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>V5_G2_RUNTIME_PACKAGE_REVIEW_ACCEPTED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -45403,7 +45516,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6103649bf962438e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00c425451a21408b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(gate): accept refreshed V5-G3 regression
</commit_message>
<xml_diff>
--- a/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
+++ b/docs/planning/TXWZS_MASTER_DEVELOPMENT_CONTROL.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="Rceab31ca3be54c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="Re1683059dc844e36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="Re2e5f96788574e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="Re2316db27f8342ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="R84389910fd8447b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="R5477667f55774b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R9ac38c5b5c304426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="R8d88adcf82f744a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="R33a2630540fd40a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Ree07b85f5e764d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="Rff3ac0300ff34991"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="R00f591e41d104392"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="Rcdb981a3e59c490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_使用说明" sheetId="1" r:id="R54f7b833efcc46ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_当前基线" sheetId="2" r:id="R876108c17a7a4876"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_长期路线图" sheetId="3" r:id="R5744b6cbd03142b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_任务总表" sheetId="4" r:id="R73f58c92a7dd4059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_依赖与阶段门" sheetId="5" r:id="Rabd602bc7de248f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_验收矩阵" sheetId="6" r:id="R34e16afc72cd4766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试矩阵" sheetId="7" r:id="R642fc1dfa5b94c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段执行记录" sheetId="8" r:id="R79c3f3777f984e09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_独立复查记录" sheetId="9" r:id="R84c75393ebc04e49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R7bfc6a7327f74b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_变更日志" sheetId="11" r:id="Ra346044488d64553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_禁止范围与保护" sheetId="12" r:id="R3135883ff0f24318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_数据对象与所有权" sheetId="13" r:id="Rbdc18dc1e0f84bc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17199,10 +17199,10 @@
     <x:t xml:space="preserve">REQ-V5-008,REQ-V5-009</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">REQ-V5-010,REQ-V5-011,REQ-V5-012</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">阶段实施时依据真实接口登记实际命令</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">REQ-V5-010,REQ-V5-011,REQ-V5-012</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">REQ-V5-006,REQ-V5-011,REQ-V5-013</x:t>
@@ -25308,7 +25308,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>1.0.2-v5-g2-fresh-review-accepted-003</x:v>
+        <x:v>1.0.3-v5-g3-refreshed-full-regression-accepted-001</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
         <x:v>6</x:v>
@@ -25327,7 +25327,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>2026-07-31</x:v>
+        <x:v>2026-08-03</x:v>
       </x:c>
       <x:c r="D6" s="9" t="s">
         <x:v>10</x:v>
@@ -25348,7 +25348,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 VERIFIED；V5 IN_PROGRESS</x:v>
+        <x:v>V4 VERIFIED / FROZEN；V5-G0 VERIFIED；V5-G1 VERIFIED；V5-G2 VERIFIED；V5-G3 VERIFIED；V5 IN_PROGRESS</x:v>
       </x:c>
       <x:c r="D7" s="9" t="s">
         <x:v>13</x:v>
@@ -25367,7 +25367,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>Post-G2 documentation convergence 已于 b1ad4a0 完成；当前唯一下一动作：M4_MIGRATION_TAG_AND_GITHUB_FRESH_CLONE_READINESS；G3+ 未启动。</x:v>
+        <x:v>V5-G3 已于 712dcbd8 的隔离运行中通过；当前唯一下一动作：WAITING_FOR_V5_G4_REAL_WINDOW_AUTHORIZATION；G4+ 未启动。</x:v>
       </x:c>
       <x:c r="D8" s="9" t="s">
         <x:v>15</x:v>
@@ -25585,7 +25585,7 @@
       </x:c>
       <x:c r="F20" s="10" t="n">
         <x:f aca="0">COUNTIFS('03_任务总表'!$C$5:$C$200,D20,'03_任务总表'!$Z$5:$Z$200,"VERIFIED")</x:f>
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="G20" s="10" t="n">
         <x:f aca="0">COUNTIFS('03_任务总表'!$C$5:$C$200,D20,'03_任务总表'!$Z$5:$Z$200,"CANCELLED")</x:f>
@@ -25593,7 +25593,7 @@
       </x:c>
       <x:c r="H20" s="16" t="n">
         <x:f aca="0">IFERROR(F20/SUMIFS('03_任务总表'!$AH$5:$AH$200,'03_任务总表'!$C$5:$C$200,D20),0)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.8409090909090909</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0">
@@ -26549,7 +26549,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f0ce5f57a7841a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra47d7cdfef2e4427"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26863,6 +26863,29 @@
         <x:v>RVW-V5-G2-003</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>1.0.3-v5-g3-refreshed-full-regression-accepted-001</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Main Codex</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>接受 refreshed V5-G3 隔离全量回归与追溯</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>V5-P4-T005、V5-P7-T001..T003、V5-G3、当前基线、测试和证据字段</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>712dcbd8 在隔离 Godot 4.5.1 下通过所有 G3 自动验收；不进入 G4-G6</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>V5-G3-R1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -26870,7 +26893,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69e535b6fc854f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcac38ff5662c49f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26926,13 +26949,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="29" t="str">
-        <x:v>V5-G2 已 fresh independently accepted；仍禁止 G3/G4/G5/G6/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
+        <x:v>V5-G3 已 refreshed regression accepted；仍禁止 G4/G5/G6/P6/V6/第二兵种/多 active/敌方 AI/围城/新战斗</x:v>
       </x:c>
       <x:c r="C5" s="7" t="str">
-        <x:v>stable-ID boundary repair 已由不同 reviewer 绑定完整提交链并独立通过；本轮只形成 acceptance checkpoint</x:v>
+        <x:v>G3 只记录隔离自动回归与追溯；不改变后续 Gate 的授权边界</x:v>
       </x:c>
       <x:c r="D5" s="29" t="str">
-        <x:v>V5-G0/G1/G2 VERIFIED；精确 16 项 runtime tasks VERIFIED；后续门保持 NOT_STARTED</x:v>
+        <x:v>V5-G0/G1/G2/G3 VERIFIED；G4-G6/P6/V6 保持 NOT_STARTED</x:v>
       </x:c>
       <x:c r="E5" s="8" t="s">
         <x:v>1555</x:v>
@@ -27081,7 +27104,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R874f37b6b1814f1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942cb42ed9894369"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27915,7 +27938,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb20830482aa442dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2b62331f27540cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28054,7 +28077,7 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>Post-G2 documentation convergence checkpoint b1ad4a09e202904aced9262104545867a97573cb；exact 8 protected S1A.2 untracked</x:v>
+        <x:v>validated source 712dcbd8e092ff844c4274a2f3a3c260d29998e7；V5-G3 refreshed full regression accepted</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
         <x:v>CONFIRMED</x:v>
@@ -28063,7 +28086,7 @@
         <x:v>git log/status + docs/reports/TXWZS_V5_G2_FINAL_ACCEPTANCE.md + protected SHA-256</x:v>
       </x:c>
       <x:c r="E10" s="19" t="str">
-        <x:v>b1ad4a0 仅含文档/规划资产；V5-G2 已独立接受；G3+ 未启动</x:v>
+        <x:v>G3 evidence is isolated/headless only; G4 real window, G5 review, and G6 user freeze remain unstarted.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" hidden="0" customHeight="1">
@@ -28137,7 +28160,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>无持续 GUI PID；正式 city/Blackstone/C0 与 editor scan 均 exit 0</x:v>
+        <x:v>无持续 GUI PID；G3 isolated city/Blackstone/C0/editor scan exit 0</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
         <x:v>CONFIRMED</x:v>
@@ -28146,7 +28169,7 @@
         <x:v>docs/reports/TXWZS_V5_G2_FINAL_ACCEPTANCE.md</x:v>
       </x:c>
       <x:c r="E15" s="10" t="str">
-        <x:v>本轮只验证 headless runtime，不进入 G4 实际窗口门</x:v>
+        <x:v>G3 does not satisfy the G4 real-window gate.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" hidden="0" customHeight="1">
@@ -28422,7 +28445,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0345e24b70aa4c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd08e0c2389054ec9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28637,7 +28660,7 @@
       </x:c>
       <x:c r="P6" s="16" t="n">
         <x:f aca="0">IFERROR(COUNTIFS('03_任务总表'!$C$5:$C$200,$A6,'03_任务总表'!$Z$5:$Z$200,"VERIFIED")/SUMIFS('03_任务总表'!$AH$5:$AH$200,'03_任务总表'!$C$5:$C$200,$A6),0)</x:f>
-        <x:v>0.75</x:v>
+        <x:v>0.8409090909090909</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="44" hidden="0" customHeight="1">
@@ -29047,7 +29070,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe6ec25910f74858"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1522737752084b77"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -32891,21 +32914,29 @@
       <x:c r="Y38" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="Z38" s="9" t="s">
-        <x:v>6</x:v>
+      <x:c r="Z38" s="9" t="str">
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA38" s="10"/>
       <x:c r="AB38" s="10"/>
       <x:c r="AC38" s="10"/>
-      <x:c r="AD38" s="10"/>
-      <x:c r="AE38" s="10"/>
-      <x:c r="AF38" s="10"/>
+      <x:c r="AD38" s="10" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="AE38" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
+      <x:c r="AF38" s="10" t="str">
+        <x:v>V5-G3-R1</x:v>
+      </x:c>
       <x:c r="AG38" s="10"/>
       <x:c r="AH38" s="23" t="n">
         <x:f aca="0">IF(AND($Z38="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG38,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AI38" s="10"/>
+      <x:c r="AI38" s="10" t="str">
+        <x:v>V5-G3 refreshed isolated regression accepted at 712dcbd8: 37/37 runners, 1819 PASS lines, focused/persistence/scene/editor evidence; G4-G6 remain NOT_STARTED.</x:v>
+      </x:c>
       <x:c r="AJ38" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -33806,21 +33837,29 @@
       <x:c r="Y47" s="9" t="s">
         <x:v>378</x:v>
       </x:c>
-      <x:c r="Z47" s="9" t="s">
-        <x:v>6</x:v>
+      <x:c r="Z47" s="9" t="str">
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA47" s="10"/>
       <x:c r="AB47" s="10"/>
       <x:c r="AC47" s="10"/>
-      <x:c r="AD47" s="10"/>
-      <x:c r="AE47" s="10"/>
-      <x:c r="AF47" s="10"/>
+      <x:c r="AD47" s="10" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="AE47" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
+      <x:c r="AF47" s="10" t="str">
+        <x:v>V5-G3-R1</x:v>
+      </x:c>
       <x:c r="AG47" s="10"/>
       <x:c r="AH47" s="23" t="n">
         <x:f aca="0">IF(AND($Z47="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG47,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AI47" s="10"/>
+      <x:c r="AI47" s="10" t="str">
+        <x:v>V5-G3 refreshed isolated regression accepted at 712dcbd8: 37/37 runners, 1819 PASS lines, focused/persistence/scene/editor evidence; G4-G6 remain NOT_STARTED.</x:v>
+      </x:c>
       <x:c r="AJ47" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -33901,21 +33940,29 @@
       <x:c r="Y48" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="Z48" s="9" t="s">
-        <x:v>6</x:v>
+      <x:c r="Z48" s="9" t="str">
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA48" s="10"/>
       <x:c r="AB48" s="10"/>
       <x:c r="AC48" s="10"/>
-      <x:c r="AD48" s="10"/>
-      <x:c r="AE48" s="10"/>
-      <x:c r="AF48" s="10"/>
+      <x:c r="AD48" s="10" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="AE48" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
+      <x:c r="AF48" s="10" t="str">
+        <x:v>V5-G3-R1</x:v>
+      </x:c>
       <x:c r="AG48" s="10"/>
       <x:c r="AH48" s="23" t="n">
         <x:f aca="0">IF(AND($Z48="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG48,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AI48" s="10"/>
+      <x:c r="AI48" s="10" t="str">
+        <x:v>V5-G3 refreshed isolated regression accepted at 712dcbd8: 37/37 runners, 1819 PASS lines, focused/persistence/scene/editor evidence; G4-G6 remain NOT_STARTED.</x:v>
+      </x:c>
       <x:c r="AJ48" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -33996,21 +34043,29 @@
       <x:c r="Y49" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="Z49" s="9" t="s">
-        <x:v>6</x:v>
+      <x:c r="Z49" s="9" t="str">
+        <x:v>VERIFIED</x:v>
       </x:c>
       <x:c r="AA49" s="10"/>
       <x:c r="AB49" s="10"/>
       <x:c r="AC49" s="10"/>
-      <x:c r="AD49" s="10"/>
-      <x:c r="AE49" s="10"/>
-      <x:c r="AF49" s="10"/>
+      <x:c r="AD49" s="10" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="AE49" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
+      <x:c r="AF49" s="10" t="str">
+        <x:v>V5-G3-R1</x:v>
+      </x:c>
       <x:c r="AG49" s="10"/>
       <x:c r="AH49" s="23" t="n">
         <x:f aca="0">IF(AND($Z49="CANCELLED",COUNTIFS('09_风险与决策'!$A$5:$A$100,$AG49,'09_风险与决策'!$B$5:$B$100,"Decision",'09_风险与决策'!$L$5:$L$100,"ACCEPTED")&gt;0),0,1)</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AI49" s="10"/>
+      <x:c r="AI49" s="10" t="str">
+        <x:v>V5-G3 refreshed isolated regression accepted at 712dcbd8: 37/37 runners, 1819 PASS lines, focused/persistence/scene/editor evidence; G4-G6 remain NOT_STARTED.</x:v>
+      </x:c>
       <x:c r="AJ49" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -38105,7 +38160,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3673d05ade124d90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35ab4cb4863b408c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38599,13 +38654,21 @@
       <x:c r="G15" s="10" t="s">
         <x:v>986</x:v>
       </x:c>
-      <x:c r="H15" s="9" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="I15" s="10"/>
-      <x:c r="J15" s="10"/>
-      <x:c r="K15" s="10"/>
-      <x:c r="L15" s="10"/>
+      <x:c r="H15" s="9" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="I15" s="10" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="J15" s="10" t="str">
+        <x:v>Main Codex</x:v>
+      </x:c>
+      <x:c r="K15" s="10" t="str">
+        <x:v>/root</x:v>
+      </x:c>
+      <x:c r="L15" s="10" t="str">
+        <x:v>TXWZS2_V5_G3_REFRESHED_FULL_REGRESSION_AND_TRACEABILITY_ACCEPTED: isolated 712dcbd8; 37/37 runners; 1819 PASS; P0-01 10/10; R2C-02 20/20; persistence 51/51; editor/scenes/diff all pass. G4-G6 remain NOT_STARTED.</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="38" hidden="0" customHeight="1">
       <x:c r="A16" s="9" t="s">
@@ -40119,7 +40182,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b63273a5e84d49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf41ebb9cafe2417e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41104,7 +41167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91473d388f974c68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63903504f3e541c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42969,20 +43032,24 @@
       <x:c r="H43" s="10" t="s">
         <x:v>616</x:v>
       </x:c>
-      <x:c r="I43" s="10" t="s">
-        <x:v>1314</x:v>
+      <x:c r="I43" s="10" t="str">
+        <x:v>Godot 4.5.1 isolated --headless --path &lt;exact archive&gt; --script res://tests/run_v5_encounter_writeback_smoke.gd</x:v>
       </x:c>
       <x:c r="J43" s="9" t="s">
         <x:v>1309</x:v>
       </x:c>
-      <x:c r="K43" s="9" t="s">
-        <x:v>1172</x:v>
-      </x:c>
-      <x:c r="L43" s="10"/>
+      <x:c r="K43" s="9" t="str">
+        <x:v>PASS_MAIN_AGENT</x:v>
+      </x:c>
+      <x:c r="L43" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
       <x:c r="M43" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="N43" s="25"/>
+      <x:c r="N43" s="25" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
       <x:c r="O43" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -43175,7 +43242,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="C48" s="9" t="s">
-        <x:v>1315</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="D48" s="9" t="s">
         <x:v>1308</x:v>
@@ -43238,7 +43305,7 @@
         <x:v>661</x:v>
       </x:c>
       <x:c r="I49" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J49" s="9" t="s">
         <x:v>1309</x:v>
@@ -43279,7 +43346,7 @@
         <x:v>670</x:v>
       </x:c>
       <x:c r="I50" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J50" s="9" t="s">
         <x:v>1309</x:v>
@@ -43320,7 +43387,7 @@
         <x:v>678</x:v>
       </x:c>
       <x:c r="I51" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J51" s="9" t="s">
         <x:v>1309</x:v>
@@ -43360,20 +43427,24 @@
       <x:c r="H52" s="10" t="s">
         <x:v>687</x:v>
       </x:c>
-      <x:c r="I52" s="10" t="s">
-        <x:v>1314</x:v>
+      <x:c r="I52" s="10" t="str">
+        <x:v>G3 isolated authority inventory + requirement/task/test traceability matrices</x:v>
       </x:c>
       <x:c r="J52" s="9" t="s">
         <x:v>1309</x:v>
       </x:c>
-      <x:c r="K52" s="9" t="s">
-        <x:v>1172</x:v>
-      </x:c>
-      <x:c r="L52" s="10"/>
+      <x:c r="K52" s="9" t="str">
+        <x:v>PASS_MAIN_AGENT</x:v>
+      </x:c>
+      <x:c r="L52" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
       <x:c r="M52" s="9" t="s">
         <x:v>378</x:v>
       </x:c>
-      <x:c r="N52" s="25"/>
+      <x:c r="N52" s="25" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
       <x:c r="O52" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -43401,20 +43472,24 @@
       <x:c r="H53" s="10" t="s">
         <x:v>694</x:v>
       </x:c>
-      <x:c r="I53" s="10" t="s">
-        <x:v>1314</x:v>
+      <x:c r="I53" s="10" t="str">
+        <x:v>G3 isolated focused runners and dynamic discovery (37/37; 1819 PASS lines)</x:v>
       </x:c>
       <x:c r="J53" s="9" t="s">
         <x:v>1309</x:v>
       </x:c>
-      <x:c r="K53" s="9" t="s">
-        <x:v>1172</x:v>
-      </x:c>
-      <x:c r="L53" s="10"/>
+      <x:c r="K53" s="9" t="str">
+        <x:v>PASS_MAIN_AGENT</x:v>
+      </x:c>
+      <x:c r="L53" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
       <x:c r="M53" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="N53" s="25"/>
+      <x:c r="N53" s="25" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
       <x:c r="O53" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -43442,20 +43517,24 @@
       <x:c r="H54" s="9" t="s">
         <x:v>700</x:v>
       </x:c>
-      <x:c r="I54" s="10" t="s">
-        <x:v>1314</x:v>
+      <x:c r="I54" s="10" t="str">
+        <x:v>G3 isolated dynamic full regression + editor/scene/import/diff/error scans</x:v>
       </x:c>
       <x:c r="J54" s="9" t="s">
         <x:v>1309</x:v>
       </x:c>
-      <x:c r="K54" s="9" t="s">
-        <x:v>1172</x:v>
-      </x:c>
-      <x:c r="L54" s="10"/>
+      <x:c r="K54" s="9" t="str">
+        <x:v>PASS_MAIN_AGENT</x:v>
+      </x:c>
+      <x:c r="L54" s="10" t="str">
+        <x:v>docs/reports/TXWZS_V5_G3_REFRESHED_FULL_REGRESSION.md; external G3 evidence package</x:v>
+      </x:c>
       <x:c r="M54" s="9" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="N54" s="25"/>
+      <x:c r="N54" s="25" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
       <x:c r="O54" s="9" t="s">
         <x:v>618</x:v>
       </x:c>
@@ -43486,7 +43565,7 @@
         <x:v>708</x:v>
       </x:c>
       <x:c r="I55" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J55" s="9" t="s">
         <x:v>1309</x:v>
@@ -43527,7 +43606,7 @@
         <x:v>715</x:v>
       </x:c>
       <x:c r="I56" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J56" s="9" t="s">
         <x:v>1309</x:v>
@@ -43568,7 +43647,7 @@
         <x:v>723</x:v>
       </x:c>
       <x:c r="I57" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J57" s="9" t="s">
         <x:v>1309</x:v>
@@ -43609,7 +43688,7 @@
         <x:v>730</x:v>
       </x:c>
       <x:c r="I58" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J58" s="9" t="s">
         <x:v>1309</x:v>
@@ -43650,7 +43729,7 @@
         <x:v>743</x:v>
       </x:c>
       <x:c r="I59" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J59" s="9" t="s">
         <x:v>1309</x:v>
@@ -43691,7 +43770,7 @@
         <x:v>753</x:v>
       </x:c>
       <x:c r="I60" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J60" s="9" t="s">
         <x:v>1309</x:v>
@@ -43732,7 +43811,7 @@
         <x:v>761</x:v>
       </x:c>
       <x:c r="I61" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J61" s="9" t="s">
         <x:v>1309</x:v>
@@ -43773,7 +43852,7 @@
         <x:v>767</x:v>
       </x:c>
       <x:c r="I62" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J62" s="9" t="s">
         <x:v>1309</x:v>
@@ -43814,7 +43893,7 @@
         <x:v>772</x:v>
       </x:c>
       <x:c r="I63" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J63" s="9" t="s">
         <x:v>1309</x:v>
@@ -43855,7 +43934,7 @@
         <x:v>777</x:v>
       </x:c>
       <x:c r="I64" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J64" s="9" t="s">
         <x:v>1309</x:v>
@@ -43896,7 +43975,7 @@
         <x:v>782</x:v>
       </x:c>
       <x:c r="I65" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J65" s="9" t="s">
         <x:v>1309</x:v>
@@ -43937,7 +44016,7 @@
         <x:v>790</x:v>
       </x:c>
       <x:c r="I66" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J66" s="9" t="s">
         <x:v>1309</x:v>
@@ -43978,7 +44057,7 @@
         <x:v>796</x:v>
       </x:c>
       <x:c r="I67" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J67" s="9" t="s">
         <x:v>1309</x:v>
@@ -44019,7 +44098,7 @@
         <x:v>803</x:v>
       </x:c>
       <x:c r="I68" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J68" s="9" t="s">
         <x:v>1309</x:v>
@@ -44060,7 +44139,7 @@
         <x:v>808</x:v>
       </x:c>
       <x:c r="I69" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J69" s="9" t="s">
         <x:v>1309</x:v>
@@ -44101,7 +44180,7 @@
         <x:v>815</x:v>
       </x:c>
       <x:c r="I70" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J70" s="9" t="s">
         <x:v>1309</x:v>
@@ -44144,7 +44223,7 @@
         <x:v>823</x:v>
       </x:c>
       <x:c r="I71" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J71" s="9" t="s">
         <x:v>1309</x:v>
@@ -44187,7 +44266,7 @@
         <x:v>829</x:v>
       </x:c>
       <x:c r="I72" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J72" s="9" t="s">
         <x:v>1309</x:v>
@@ -44228,7 +44307,7 @@
         <x:v>836</x:v>
       </x:c>
       <x:c r="I73" s="10" t="s">
-        <x:v>1314</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="J73" s="9" t="s">
         <x:v>1309</x:v>
@@ -44275,7 +44354,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0d2d0bfbe74220"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7cd46ce504a4ca6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44686,6 +44765,50 @@
       </x:c>
       <x:c r="N11" t="str">
         <x:v>No；do not enter G3/push/deploy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>RUN-V5-G3-R1-REFRESHED-REGRESSION</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Main Codex / GPT-5.6 Terra high</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>V5-P4-T005,V5-P7-T001,V5-P7-T002,V5-P7-T003</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>712dcbd8; clean; no nonignored untracked</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>documentation and planning record only after isolated verification</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>exact git archive + sandboxed Godot 4.5.1 + dynamic runner discovery + focused/persistence + editor/scenes + authority/diff/traceability audits</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>37/37 dynamic; 1819 PASS; P0-01 10/10; R2C-02 20/20; V5 persistence 51/51</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>G4 real window, G5 review, G6 user freeze, R2C-03, and V6 remain unstarted</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>documentation-only gate record commit; source tree unchanged</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>docs(gate): accept refreshed V5-G3 regression</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>WAITING_FOR_V5_G4_REAL_WINDOW_AUTHORIZATION</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>G4 requires separate real-window authorization</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -44718,7 +44841,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0385ac24585f4a49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b1b354bd1934526"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -45159,7 +45282,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcde35068a3cb4e40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafae96c6240b424b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>